<commit_message>
feat: apply validated Ubidots sync proposals safely
</commit_message>
<xml_diff>
--- a/registros.xlsx
+++ b/registros.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA877"/>
+  <dimension ref="A1:AA879"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -48374,9 +48374,151 @@
         <v>{"Hora":"05:25","Observaciones":"Ningúna ","Fecha":"2026-09-08","PlacaCisterna":"0","Encargado":"Edison Giraldo Isaza"}</v>
       </c>
     </row>
+    <row r="878">
+      <c r="A878">
+        <v>44</v>
+      </c>
+      <c r="B878">
+        <v>100</v>
+      </c>
+      <c r="C878">
+        <v>19</v>
+      </c>
+      <c r="D878">
+        <v>93</v>
+      </c>
+      <c r="E878">
+        <v>110</v>
+      </c>
+      <c r="F878">
+        <v>22</v>
+      </c>
+      <c r="G878">
+        <v>14826</v>
+      </c>
+      <c r="H878" t="str">
+        <v>Uzn256</v>
+      </c>
+      <c r="I878">
+        <v>115</v>
+      </c>
+      <c r="J878">
+        <v>56</v>
+      </c>
+      <c r="K878">
+        <v>110</v>
+      </c>
+      <c r="L878">
+        <v>10</v>
+      </c>
+      <c r="O878" t="str">
+        <v>Inicia trasiego</v>
+      </c>
+      <c r="P878" t="str">
+        <v>Jorge mario Cadavid gallego</v>
+      </c>
+      <c r="Q878" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="R878" t="str">
+        <v>06:14:00</v>
+      </c>
+      <c r="U878">
+        <v>1788873375834</v>
+      </c>
+      <c r="V878" t="str">
+        <v>2026-09-08T13:16:15.834Z</v>
+      </c>
+      <c r="W878" t="str">
+        <v>08/09/2026, 08:16:15</v>
+      </c>
+      <c r="X878">
+        <v>122</v>
+      </c>
+      <c r="Y878">
+        <v>11</v>
+      </c>
+      <c r="Z878">
+        <v>11</v>
+      </c>
+      <c r="AA878" t="str">
+        <v>{"Encargado":"Jorge mario Cadavid gallego","Hora":"06:14","Observaciones":"Inicia trasiego","PlacaCisterna":"Uzn256","Fecha":"2026-09-08"}</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879">
+        <v>85</v>
+      </c>
+      <c r="B879">
+        <v>100</v>
+      </c>
+      <c r="C879">
+        <v>19</v>
+      </c>
+      <c r="D879">
+        <v>44</v>
+      </c>
+      <c r="E879">
+        <v>110</v>
+      </c>
+      <c r="F879">
+        <v>22</v>
+      </c>
+      <c r="G879">
+        <v>14826</v>
+      </c>
+      <c r="H879" t="str">
+        <v>Uzn256</v>
+      </c>
+      <c r="I879">
+        <v>115</v>
+      </c>
+      <c r="J879">
+        <v>56</v>
+      </c>
+      <c r="K879">
+        <v>110</v>
+      </c>
+      <c r="L879">
+        <v>12</v>
+      </c>
+      <c r="O879" t="str">
+        <v>Termina trasiego</v>
+      </c>
+      <c r="P879" t="str">
+        <v>Jorge mario Cadavid gallego</v>
+      </c>
+      <c r="Q879" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="R879" t="str">
+        <v>08:16:00</v>
+      </c>
+      <c r="U879">
+        <v>1788873500263</v>
+      </c>
+      <c r="V879" t="str">
+        <v>2026-09-08T13:18:20.263Z</v>
+      </c>
+      <c r="W879" t="str">
+        <v>08/09/2026, 08:18:20</v>
+      </c>
+      <c r="X879">
+        <v>2</v>
+      </c>
+      <c r="Y879">
+        <v>11</v>
+      </c>
+      <c r="Z879">
+        <v>11</v>
+      </c>
+      <c r="AA879" t="str">
+        <v>{"PlacaCisterna":"Uzn256","Hora":"08:16","Encargado":"Jorge mario Cadavid gallego","Observaciones":"Termina trasiego","Fecha":"2026-09-08"}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA877"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA879"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
data: sync latest validated Ubidots record
</commit_message>
<xml_diff>
--- a/registros.xlsx
+++ b/registros.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA879"/>
+  <dimension ref="A1:AA880"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -48516,9 +48516,80 @@
         <v>{"PlacaCisterna":"Uzn256","Hora":"08:16","Encargado":"Jorge mario Cadavid gallego","Observaciones":"Termina trasiego","Fecha":"2026-09-08"}</v>
       </c>
     </row>
+    <row r="880">
+      <c r="A880">
+        <v>66</v>
+      </c>
+      <c r="B880">
+        <v>100</v>
+      </c>
+      <c r="C880">
+        <v>19</v>
+      </c>
+      <c r="D880">
+        <v>44</v>
+      </c>
+      <c r="E880">
+        <v>110</v>
+      </c>
+      <c r="F880">
+        <v>22</v>
+      </c>
+      <c r="G880">
+        <v>14826</v>
+      </c>
+      <c r="H880" t="str">
+        <v>Uzn256</v>
+      </c>
+      <c r="I880">
+        <v>110</v>
+      </c>
+      <c r="J880">
+        <v>56</v>
+      </c>
+      <c r="K880">
+        <v>110</v>
+      </c>
+      <c r="L880">
+        <v>12</v>
+      </c>
+      <c r="O880" t="str">
+        <v>Ninguna</v>
+      </c>
+      <c r="P880" t="str">
+        <v>Jorge mario Cadavid gallego</v>
+      </c>
+      <c r="Q880" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="R880" t="str">
+        <v>13:16:00</v>
+      </c>
+      <c r="U880">
+        <v>1788891488888</v>
+      </c>
+      <c r="V880" t="str">
+        <v>2026-09-08T18:18:08.888Z</v>
+      </c>
+      <c r="W880" t="str">
+        <v>08/09/2026, 13:18:08</v>
+      </c>
+      <c r="X880">
+        <v>2</v>
+      </c>
+      <c r="Y880">
+        <v>11</v>
+      </c>
+      <c r="Z880">
+        <v>11</v>
+      </c>
+      <c r="AA880" t="str">
+        <v>{"Encargado":"Jorge mario Cadavid gallego","Fecha":"2026-09-08","Hora":"13:16","Observaciones":"Ninguna","PlacaCisterna":"Uzn256"}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA879"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA880"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>